<commit_message>
Add tests for Excel field extraction and output formatting
- Implemented a test suite in `test_split_output.py` to validate the functionality of the ExcelFieldExtractor.
- Created test Excel files with both empty and non-empty tables to ensure accurate field extraction.
- Added assertions to verify the structure of the JSON output generated from the extraction process.
- Included two new Excel files: `test_error_logging.xlsx` and `test_incomplete_rows.xlsx` for further testing scenarios.
</commit_message>
<xml_diff>
--- a/test_output/realistic_test_result.xlsx
+++ b/test_output/realistic_test_result.xlsx
@@ -436,14 +436,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="100" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,11 +463,6 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>字段列表</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
           <t>字段+示例</t>
         </is>
       </c>
@@ -488,11 +482,6 @@
         <v>4</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>level_name, level_desc, difficulty, reward_desc</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>level_name,新手村, level_desc,这是新手村的关卡，难度简单, difficulty,简单, reward_desc,获得100金币和经验</t>
         </is>

</xml_diff>